<commit_message>
Versión final del sistema de recibos`
</commit_message>
<xml_diff>
--- a/datos-empresa.xlsx
+++ b/datos-empresa.xlsx
@@ -1,22 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr/>
   <bookViews>
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Recibos" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Comprobantes" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Configuracion" state="visible" r:id="rId6"/>
+    <sheet name="Recibos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Comprobantes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Configuracion" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Fecha</t>
   </si>
@@ -36,16 +38,16 @@
     <t>12/3/2026</t>
   </si>
   <si>
-    <t>HUGO MARTIN VILLALBA</t>
-  </si>
-  <si>
-    <t>[{"cant":"1","desc":"servicio de promotor de seguros","precio":"05000"}]</t>
+    <t xml:space="preserve">HUGO MARTIN VILLALBA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[{"cant":"1","desc":"servicio de promotor de seguros","precio":"05000"}]</t>
   </si>
   <si>
     <t>$5000.00</t>
   </si>
   <si>
-    <t>villalba hugo</t>
+    <t xml:space="preserve">villalba hugo</t>
   </si>
   <si>
     <t>[{"cant":"1","desc":"prueba","precio":"50000"}]</t>
@@ -54,46 +56,46 @@
     <t>$50000.00</t>
   </si>
   <si>
-    <t>hugo villalba</t>
-  </si>
-  <si>
-    <t>[{"cant":"1","desc":"producos  de seguros","precio":"05000"}]</t>
-  </si>
-  <si>
-    <t>NUEVO CLIENTE</t>
-  </si>
-  <si>
-    <t>[{"cant":"1","desc":"POROTROS SEGUROS","precio":"010000"}]</t>
+    <t xml:space="preserve">hugo villalba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[{"cant":"1","desc":"producos  de seguros","precio":"05000"}]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NUEVO CLIENTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[{"cant":"1","desc":"POROTROS SEGUROS","precio":"010000"}]</t>
   </si>
   <si>
     <t>$10000.00</t>
   </si>
   <si>
-    <t>NUEVO CLENTE NUEVO</t>
+    <t xml:space="preserve">NUEVO CLENTE NUEVO</t>
   </si>
   <si>
     <t>[{"cant":"1","desc":"SEGUROS","precio":"10000"}]</t>
   </si>
   <si>
-    <t>NUEVO CLENTE NUEVO 2</t>
-  </si>
-  <si>
-    <t>[{"cant":"1","desc":"seguros nuevos","precio":"07000"}]</t>
+    <t xml:space="preserve">NUEVO CLENTE NUEVO 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[{"cant":"1","desc":"seguros nuevos","precio":"07000"}]</t>
   </si>
   <si>
     <t>$7000.00</t>
   </si>
   <si>
-    <t>clinte cinco</t>
-  </si>
-  <si>
-    <t>[{"cant":"1","desc":"segurtos varios","precio":"020000"}]</t>
+    <t xml:space="preserve">clinte cinco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[{"cant":"1","desc":"segurtos varios","precio":"020000"}]</t>
   </si>
   <si>
     <t>$20000.00</t>
   </si>
   <si>
-    <t>ultimo cliente</t>
+    <t xml:space="preserve">ultimo cliente</t>
   </si>
   <si>
     <t>[{"cant":"1","desc":"seguros","precio":"015000"}]</t>
@@ -108,13 +110,13 @@
     <t>Empresa</t>
   </si>
   <si>
-    <t>HALIER NATALIA SOLEDAD</t>
+    <t xml:space="preserve">HALIER NATALIA SOLEDAD</t>
   </si>
   <si>
     <t>Direccion</t>
   </si>
   <si>
-    <t>YUNKA 540</t>
+    <t xml:space="preserve">YUNKA 540</t>
   </si>
   <si>
     <t>Telefono</t>
@@ -132,26 +134,25 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="3">
     <font>
+      <sz val="11.000000"/>
       <color theme="1"/>
-      <family val="2"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="11.000000"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11.000000"/>
       <color theme="10"/>
-      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -163,14 +164,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="1">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -180,12 +174,12 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -682,18 +676,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="13.00390625" customWidth="1"/>
-    <col min="2" max="2" width="13.28125" customWidth="1"/>
-    <col min="3" max="3" width="54.140625" customWidth="1"/>
-    <col min="4" max="4" width="49.57421875" customWidth="1"/>
-    <col min="5" max="5" width="15.28125" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="13.00390625"/>
+    <col customWidth="1" min="2" max="2" width="13.28125"/>
+    <col customWidth="1" min="3" max="3" width="54.140625"/>
+    <col customWidth="1" min="4" max="4" width="49.57421875"/>
+    <col customWidth="1" min="5" max="5" width="15.28125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -710,7 +703,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -727,7 +720,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -744,7 +737,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -761,7 +754,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -778,7 +771,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -795,7 +788,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -812,7 +805,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -829,7 +822,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -847,47 +840,49 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="600" verticalDpi="600" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" usePrinterDefaults="1" copies="1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="19.140625" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="19.140625"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.25" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" ht="14.25" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" ht="14.25" customHeight="1">
       <c r="A2">
         <v>108</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="600" verticalDpi="600" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" usePrinterDefaults="1" copies="1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:B5"/>
-  <sheetFormatPr defaultRowHeight="14.25" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" customHeight="1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetFormatPr defaultRowHeight="14.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="37.421875" customWidth="1"/>
-    <col min="2" max="2" width="49.140625" customWidth="1"/>
-    <col min="3" max="3" width="20.28125" customWidth="1"/>
-    <col min="4" max="4" width="45.421875" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="37.421875"/>
+    <col customWidth="1" min="2" max="2" width="49.140625"/>
+    <col customWidth="1" min="3" max="3" width="20.28125"/>
+    <col customWidth="1" min="4" max="4" width="45.421875"/>
   </cols>
   <sheetData>
-    <row r="2" ht="14.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>29</v>
       </c>
@@ -895,7 +890,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" ht="14.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>31</v>
       </c>
@@ -903,7 +898,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" ht="14.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>33</v>
       </c>
@@ -911,7 +906,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="5" ht="14.25" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>35</v>
       </c>
@@ -921,9 +916,11 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId1"/>
+    <hyperlink r:id="rId1" ref="B5"/>
   </hyperlinks>
-  <pageMargins left="0.7007874015748032" right="0.7007874015748032" top="0.7519685039370079" bottom="0.7519685039370079" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="600" verticalDpi="600" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" usePrinterDefaults="1" copies="1"/>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>